<commit_message>
fix: Direct VPS PostgreSQL IP connection 188.132.198.144
</commit_message>
<xml_diff>
--- a/personeller.xlsx
+++ b/personeller.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\PRJrms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{15BA1481-3EE2-47F2-B16D-6F58305F7393}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F866A925-EB58-4965-82E5-B706FBBF0C64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="20700" windowHeight="11140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="20700" windowHeight="11140" tabRatio="623" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Personeller" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="63">
   <si>
     <t>Ad</t>
   </si>
@@ -115,12 +115,6 @@
     <t>'+905337661142</t>
   </si>
   <si>
-    <t>Yedek</t>
-  </si>
-  <si>
-    <t>gomisenseapp@gmail.com</t>
-  </si>
-  <si>
     <t>'+905448411142</t>
   </si>
   <si>
@@ -160,12 +154,6 @@
     <t>'+905511084284</t>
   </si>
   <si>
-    <t xml:space="preserve">Test Kullanıcı </t>
-  </si>
-  <si>
-    <t>test59@gmail.com</t>
-  </si>
-  <si>
     <t>Süleyman</t>
   </si>
   <si>
@@ -197,16 +185,48 @@
   </si>
   <si>
     <t>duranalperen1905@gmail.com</t>
+  </si>
+  <si>
+    <t>şifre</t>
+  </si>
+  <si>
+    <t>Rol</t>
+  </si>
+  <si>
+    <t>üye</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>gamzevardar@suitablepos.com</t>
+  </si>
+  <si>
+    <t>Gamze</t>
+  </si>
+  <si>
+    <t>Vardar</t>
+  </si>
+  <si>
+    <t>+905524685391</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -229,13 +249,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Köprü" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -573,16 +597,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="2" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="30.83203125" customWidth="1"/>
+    <col min="5" max="5" width="13.75" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -590,13 +615,19 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -604,13 +635,19 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2">
+        <v>123456</v>
+      </c>
+      <c r="F2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -618,13 +655,19 @@
         <v>9</v>
       </c>
       <c r="C3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3">
+        <v>123456</v>
+      </c>
+      <c r="F3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -632,13 +675,19 @@
         <v>13</v>
       </c>
       <c r="C4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D4" t="s">
         <v>14</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4">
+        <v>123456</v>
+      </c>
+      <c r="F4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -646,13 +695,19 @@
         <v>17</v>
       </c>
       <c r="C5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" t="s">
         <v>18</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5">
+        <v>123456</v>
+      </c>
+      <c r="F5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -660,13 +715,19 @@
         <v>21</v>
       </c>
       <c r="C6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" t="s">
         <v>22</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6">
+        <v>123456</v>
+      </c>
+      <c r="F6" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -674,13 +735,19 @@
         <v>21</v>
       </c>
       <c r="C7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" t="s">
         <v>25</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7">
+        <v>123456</v>
+      </c>
+      <c r="F7" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>27</v>
       </c>
@@ -688,142 +755,185 @@
         <v>28</v>
       </c>
       <c r="C8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" t="s">
         <v>29</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8">
+        <v>123456</v>
+      </c>
+      <c r="F8" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9">
+        <v>1453</v>
+      </c>
+      <c r="F9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10">
+        <v>123456</v>
+      </c>
+      <c r="F10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" t="s">
+        <v>57</v>
+      </c>
+      <c r="D11" t="s">
+        <v>42</v>
+      </c>
+      <c r="E11">
+        <v>123456</v>
+      </c>
+      <c r="F11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" t="s">
+        <v>57</v>
+      </c>
+      <c r="D12" t="s">
+        <v>46</v>
+      </c>
+      <c r="E12">
+        <v>123456</v>
+      </c>
+      <c r="F12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E13">
+        <v>123456</v>
+      </c>
+      <c r="F13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>12</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" t="s">
+        <v>53</v>
+      </c>
+      <c r="E14">
+        <v>123456</v>
+      </c>
+      <c r="F14" t="s">
         <v>31</v>
       </c>
-      <c r="C9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>34</v>
-      </c>
-      <c r="B10" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D11" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>42</v>
-      </c>
-      <c r="B12" t="s">
-        <v>43</v>
-      </c>
-      <c r="C12" t="s">
-        <v>44</v>
-      </c>
-      <c r="D12" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>46</v>
-      </c>
-      <c r="B13" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" t="s">
-        <v>47</v>
-      </c>
-      <c r="D13" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>48</v>
-      </c>
-      <c r="B14" t="s">
-        <v>49</v>
-      </c>
-      <c r="C14" t="s">
-        <v>50</v>
-      </c>
-      <c r="D14" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="B15" t="s">
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="C15" t="s">
+        <v>57</v>
+      </c>
+      <c r="D15" t="s">
         <v>54</v>
       </c>
-      <c r="D15" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E15">
+        <v>123456</v>
+      </c>
+      <c r="F15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="B16" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C16" t="s">
         <v>57</v>
       </c>
-      <c r="D16" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>20</v>
-      </c>
-      <c r="B17" t="s">
-        <v>21</v>
-      </c>
-      <c r="C17" t="s">
-        <v>58</v>
-      </c>
-      <c r="D17" t="s">
-        <v>23</v>
+      <c r="D16" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E16">
+        <v>123456</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D16" r:id="rId1" xr:uid="{D1DE683B-BB3A-4918-810F-3DCA814B9A3B}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:A17 B1:D17" numberStoredAsText="1"/>
+    <ignoredError sqref="F1:F15 D1:D15 A1:B15" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>